<commit_message>
LLM Depreciation Alert test-local-test-7
</commit_message>
<xml_diff>
--- a/Scheduler_Testing.xlsx
+++ b/Scheduler_Testing.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="46">
   <si>
     <t>ProjectName</t>
   </si>
@@ -25,12 +25,15 @@
     <t>SubModule</t>
   </si>
   <si>
-    <t>LLMModel</t>
+    <t>Model</t>
   </si>
   <si>
     <t>DepreciationDate</t>
   </si>
   <si>
+    <t>Notified</t>
+  </si>
+  <si>
     <t>RecipientEmail</t>
   </si>
   <si>
@@ -49,13 +52,10 @@
     <t>us.anthropic.claude-sonnet-4-20250514-v1:0</t>
   </si>
   <si>
-    <t>samuel.k@capestart.com</t>
+    <t>amuthalingeswaran.chandrabose@capestart.com</t>
   </si>
   <si>
     <t>Protocol Docx</t>
-  </si>
-  <si>
-    <t>amuthalingeswaran.chandrabose@capestart.com</t>
   </si>
   <si>
     <t>Gowri Sankar</t>
@@ -225,7 +225,7 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="15" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
@@ -240,11 +240,11 @@
     <xf xfId="0" numFmtId="15" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -563,7 +563,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="10" width="12.719285714285713" customWidth="1" bestFit="1"/>
@@ -571,8 +571,9 @@
     <col min="3" max="3" style="12" width="34.43357142857143" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="11" width="39.71928571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="13" width="19.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="11" width="42.86214285714286" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="42.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -591,58 +592,63 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="6">
         <v>46217</v>
       </c>
-      <c r="F2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="8"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E3" s="6">
         <v>46217</v>
       </c>
-      <c r="F3" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="8"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>14</v>
@@ -650,20 +656,21 @@
       <c r="C4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="7" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="6">
         <v>46217</v>
       </c>
-      <c r="F4" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="8"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>14</v>
@@ -671,20 +678,21 @@
       <c r="C5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="6">
         <v>46217</v>
       </c>
-      <c r="F5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="8"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>18</v>
@@ -692,20 +700,21 @@
       <c r="C6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>10</v>
+      <c r="D6" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E6" s="6">
         <v>46217</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="8"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>18</v>
@@ -713,20 +722,21 @@
       <c r="C7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>10</v>
+      <c r="D7" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E7" s="6">
         <v>46217</v>
       </c>
-      <c r="F7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="8"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>21</v>
@@ -734,20 +744,21 @@
       <c r="C8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>10</v>
+      <c r="D8" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E8" s="6">
         <v>46217</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="8"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>21</v>
@@ -755,20 +766,21 @@
       <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="6">
         <v>46217</v>
       </c>
-      <c r="F9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="8"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>18</v>
@@ -776,20 +788,21 @@
       <c r="C10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="7" t="s">
         <v>26</v>
       </c>
       <c r="E10" s="6">
         <v>46217</v>
       </c>
-      <c r="F10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="8"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>18</v>
@@ -797,20 +810,21 @@
       <c r="C11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="7" t="s">
         <v>26</v>
       </c>
       <c r="E11" s="6">
         <v>46217</v>
       </c>
-      <c r="F11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="8"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>28</v>
@@ -818,20 +832,21 @@
       <c r="C12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="7" t="s">
         <v>30</v>
       </c>
       <c r="E12" s="6">
         <v>46217</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="8"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>28</v>
@@ -839,20 +854,21 @@
       <c r="C13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="7" t="s">
         <v>16</v>
       </c>
       <c r="E13" s="6">
         <v>46217</v>
       </c>
-      <c r="F13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="8"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>31</v>
@@ -860,20 +876,21 @@
       <c r="C14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E14" s="6">
         <v>46217</v>
       </c>
-      <c r="F14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="8"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>28</v>
@@ -881,20 +898,21 @@
       <c r="C15" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="7" t="s">
         <v>34</v>
       </c>
       <c r="E15" s="6">
         <v>46217</v>
       </c>
-      <c r="F15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="8"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>18</v>
@@ -902,20 +920,21 @@
       <c r="C16" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>10</v>
+      <c r="D16" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E16" s="6">
         <v>46217</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="8"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>31</v>
@@ -923,20 +942,21 @@
       <c r="C17" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="8" t="s">
-        <v>10</v>
+      <c r="D17" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E17" s="6">
         <v>46217</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="8"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B18" s="9" t="s">
         <v>37</v>
@@ -944,20 +964,21 @@
       <c r="C18" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="7" t="s">
         <v>39</v>
       </c>
       <c r="E18" s="6">
         <v>46217</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="8"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H18" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="15.75">
       <c r="A19" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>40</v>
@@ -965,20 +986,21 @@
       <c r="C19" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="8" t="s">
-        <v>10</v>
+      <c r="D19" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E19" s="6">
         <v>46217</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="8"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="15.75">
       <c r="A20" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>42</v>
@@ -986,20 +1008,21 @@
       <c r="C20" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="8" t="s">
+      <c r="D20" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E20" s="6">
         <v>46217</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="8"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="15.75">
       <c r="A21" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>14</v>
@@ -1007,35 +1030,37 @@
       <c r="C21" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E21" s="6">
         <v>46217</v>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="8"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H21" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="15.75">
       <c r="A22" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B22" s="8"/>
+        <v>8</v>
+      </c>
+      <c r="B22" s="7"/>
       <c r="C22" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="7" t="s">
         <v>24</v>
       </c>
       <c r="E22" s="6">
         <v>46217</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="8"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H22" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LLM Depreciation Alert test-local-test-8
</commit_message>
<xml_diff>
--- a/Scheduler_Testing.xlsx
+++ b/Scheduler_Testing.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="47">
   <si>
     <t>ProjectName</t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>us.anthropic.claude-sonnet-4-20250514-v1:0</t>
+  </si>
+  <si>
+    <t>2026-07-14</t>
   </si>
   <si>
     <t>amuthalingeswaran.chandrabose@capestart.com</t>
@@ -237,7 +240,7 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="15" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -615,12 +618,12 @@
       <c r="D2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="6">
-        <v>46217</v>
+      <c r="E2" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F2" s="7"/>
       <c r="G2" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H2" s="7"/>
     </row>
@@ -632,17 +635,17 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6">
-        <v>46217</v>
+      <c r="E3" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F3" s="7"/>
       <c r="G3" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H3" s="7"/>
     </row>
@@ -651,20 +654,20 @@
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="6">
-        <v>46217</v>
+        <v>17</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F4" s="7"/>
       <c r="G4" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H4" s="7"/>
     </row>
@@ -673,20 +676,20 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="6">
-        <v>46217</v>
+      <c r="E5" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H5" s="7"/>
     </row>
@@ -695,20 +698,20 @@
         <v>8</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="6">
-        <v>46217</v>
+      <c r="E6" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H6" s="7"/>
     </row>
@@ -717,20 +720,20 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="6">
-        <v>46217</v>
+      <c r="E7" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F7" s="7"/>
       <c r="G7" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H7" s="7"/>
     </row>
@@ -739,20 +742,20 @@
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="6">
-        <v>46217</v>
+      <c r="E8" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H8" s="7"/>
     </row>
@@ -761,20 +764,20 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="6">
-        <v>46217</v>
+        <v>25</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F9" s="7"/>
       <c r="G9" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H9" s="7"/>
     </row>
@@ -783,20 +786,20 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="6">
-        <v>46217</v>
+        <v>27</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F10" s="7"/>
       <c r="G10" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H10" s="7"/>
     </row>
@@ -805,20 +808,20 @@
         <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="6">
-        <v>46217</v>
+      <c r="E11" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F11" s="7"/>
       <c r="G11" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H11" s="7"/>
     </row>
@@ -827,20 +830,20 @@
         <v>8</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="6">
-        <v>46217</v>
+        <v>31</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F12" s="7"/>
       <c r="G12" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H12" s="7"/>
     </row>
@@ -849,20 +852,20 @@
         <v>8</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="6">
-        <v>46217</v>
+        <v>17</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F13" s="7"/>
       <c r="G13" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H13" s="7"/>
     </row>
@@ -871,20 +874,20 @@
         <v>8</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="6">
-        <v>46217</v>
+        <v>25</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F14" s="7"/>
       <c r="G14" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H14" s="7"/>
     </row>
@@ -893,20 +896,20 @@
         <v>8</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="6">
-        <v>46217</v>
+        <v>35</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F15" s="7"/>
       <c r="G15" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H15" s="7"/>
     </row>
@@ -915,20 +918,20 @@
         <v>8</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E16" s="6">
-        <v>46217</v>
+      <c r="E16" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F16" s="7"/>
       <c r="G16" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H16" s="7"/>
     </row>
@@ -937,20 +940,20 @@
         <v>8</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="6">
-        <v>46217</v>
+      <c r="E17" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F17" s="7"/>
       <c r="G17" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H17" s="7"/>
     </row>
@@ -959,20 +962,20 @@
         <v>8</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="6">
-        <v>46217</v>
+        <v>40</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H18" s="7"/>
     </row>
@@ -981,20 +984,20 @@
         <v>8</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E19" s="6">
-        <v>46217</v>
+      <c r="E19" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H19" s="7"/>
     </row>
@@ -1003,20 +1006,20 @@
         <v>8</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="6">
-        <v>46217</v>
+        <v>25</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F20" s="7"/>
       <c r="G20" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H20" s="7"/>
     </row>
@@ -1025,20 +1028,20 @@
         <v>8</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E21" s="6">
-        <v>46217</v>
+        <v>25</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F21" s="7"/>
       <c r="G21" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H21" s="7"/>
     </row>
@@ -1048,17 +1051,17 @@
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E22" s="6">
-        <v>46217</v>
+        <v>25</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H22" s="7"/>
     </row>

</xml_diff>